<commit_message>
adds updated data files, creates updated cleaned data files
</commit_message>
<xml_diff>
--- a/data-raw/lower_feather_release.xlsx
+++ b/data-raw/lower_feather_release.xlsx
@@ -10,7 +10,7 @@
     <sheet sheetId="1" r:id="rId1" name="lower_feather_release"/>
   </sheets>
   <definedNames>
-    <definedName name="lower_feather_release">'lower_feather_release'!$A$1:$N$33</definedName>
+    <definedName name="lower_feather_release">'lower_feather_release'!$A$1:$N$34</definedName>
   </definedNames>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
@@ -347,7 +347,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row outlineLevel="0" r="1">
@@ -2341,6 +2341,63 @@
         </is>
       </c>
     </row>
+    <row outlineLevel="0" r="34">
+      <c r="A34" s="0">
+        <v>12</v>
+      </c>
+      <c r="B34" s="0">
+        <v>288</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Chinook salmon</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Fall</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>Natural</t>
+        </is>
+      </c>
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>Lower Feather River Release Site</t>
+        </is>
+      </c>
+      <c r="H34" s="0">
+        <v>1764</v>
+      </c>
+      <c r="I34" s="1">
+        <v>46031.4779050926</v>
+      </c>
+      <c r="J34" s="0">
+        <v>7</v>
+      </c>
+      <c r="K34" s="0" t="inlineStr">
+        <is>
+          <t>Pigment / dye</t>
+        </is>
+      </c>
+      <c r="L34" s="0" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="M34" s="0" t="inlineStr">
+        <is>
+          <t>Whole body</t>
+        </is>
+      </c>
+      <c r="N34" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>